<commit_message>
feat: implement subscription management feature with backend plans logic, frontend UI, tests, and splash screen flow
</commit_message>
<xml_diff>
--- a/vapt/VAPT Requirement.xlsx
+++ b/vapt/VAPT Requirement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pthakurta/Desktop/Desktop/Aguna Solutions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E\medikto\vapt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F64FFAF-500A-BE45-ADCD-5956B218A403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2506A2E0-623D-4CAC-9249-1311502D3516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="2320" windowWidth="25800" windowHeight="15940" xr2:uid="{4F991FB9-5135-6F4B-97B9-EE2505A382D3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4F991FB9-5135-6F4B-97B9-EE2505A382D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Sr Num</t>
   </si>
@@ -62,44 +62,40 @@
     <t>Conformity Assessment</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify if agreed and identified vulnerabilities are properly closed </t>
-  </si>
-  <si>
-    <t>Ex:
-Up to 12 Ips
-IPs     05 Internal
-Ips     07 External</t>
-  </si>
-  <si>
-    <t>Ex: 
-Upto 500 Internal Ips</t>
-  </si>
-  <si>
-    <t>Ex:
-Up to 04 network devices/components
-01 Firewall
-01 WLC (Aruba OS)
-01 Switch (Aruba)</t>
-  </si>
-  <si>
     <t>Total Number of Site</t>
   </si>
   <si>
-    <t>Ex: 3</t>
-  </si>
-  <si>
     <t>Cloud, On-Prem, Hybrid (Total number of Cloud Ex: AWS, GCP etc</t>
   </si>
   <si>
     <t>Any other information</t>
   </si>
   <si>
-    <t xml:space="preserve">Please provide any relevant information </t>
-  </si>
-  <si>
-    <t>Ex:
-Number of User roles
-02 Web Applications having up to 50 pages each</t>
+    <t>External IP / Domain: api-prd.medikto.com, admin.medikto.com, medikto.health (1 Server Instance / AWS EC2).</t>
+  </si>
+  <si>
+    <t>1 AWS Cloud Region (ap-south-1 Mumbai).</t>
+  </si>
+  <si>
+    <t>Cloud (AWS) — 1 AWS EC2 instance (Docker host), 1 AWS DocumentDB cluster, 1 AWS S3 bucket.</t>
+  </si>
+  <si>
+    <t>1 External Public Elastic IP (AWS EC2 hosting Reverse Proxy).</t>
+  </si>
+  <si>
+    <t>2 Web Applications:
+1. Super Admin &amp; Hospital Admin Portal (https://admin.medikto.com ~14 pages, 3 roles)
+2. Landing Marketing Site (https://medikto.health 1 landing page).
++ REST API backend (~28 endpoints including PhonePe payment webhooks).</t>
+  </si>
+  <si>
+    <t>Review of Host Nginx SSL/TLS configuration, Docker container isolation, AWS Security Groups, and AWS S3 Bucket Policies.</t>
+  </si>
+  <si>
+    <t>Verification &amp; 1 re-test cycle after developers patch identified vulnerabilities.</t>
+  </si>
+  <si>
+    <t>Mobile Apps (Android APK + iOS TestFlight) built with Flutter; API uses JWT authentication, PhonePe Payment Gateway (S2S webhooks), and AWS DocumentDB with TLS encryption.</t>
   </si>
 </sst>
 </file>
@@ -630,14 +626,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F4453A-5DEE-CD4A-BCDE-9D4D041DF846}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.1640625" customWidth="1"/>
+    <col min="1" max="1" width="17.125" customWidth="1"/>
     <col min="2" max="2" width="26.5" customWidth="1"/>
-    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="3" max="3" width="29.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="29" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="31.5" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -648,7 +644,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="46" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="102.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -656,30 +652,32 @@
         <v>3</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="9">
         <v>2</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="67" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:3" ht="81.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="9">
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="10"/>
-    </row>
-    <row r="5" spans="1:3" ht="103" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="102.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6">
         <v>3</v>
       </c>
@@ -687,10 +685,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="119" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="119.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="6">
         <v>4</v>
       </c>
@@ -698,10 +696,10 @@
         <v>5</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="133" thickBot="1" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="122.25" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="6">
         <v>5</v>
       </c>
@@ -709,10 +707,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="89" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="89.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="6">
         <v>6</v>
       </c>
@@ -720,53 +718,53 @@
         <v>7</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="58" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="57.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="6">
         <v>7</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
     </row>

</xml_diff>